<commit_message>
Add Refresh and Add Collection Sheet actions to TPL
Tbl:DOC_Action now has 3 actions:
1. output_to_obsidian - Export YAML frontmatter to Obsidian
2. refresh_document_list - Derive doc_type_prefix (VLOOKUP),
   document_id, set created/updated/version defaults
3. add_collection_sheet - Create new Collection from TPL

Macro-based refresh chosen over pre-formatted 200 rows to
preserve copy-paste flexibility and reduce file size.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/DocumentBase_v0.1.0.xlsx
+++ b/excel/DocumentBase_v0.1.0.xlsx
@@ -9,7 +9,7 @@
     <sheet name="TPL_DOC-CATEGORY-SEQ" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -33,11 +33,17 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="游ゴシック"/>
+      <charset val="128"/>
+      <family val="3"/>
       <b val="1"/>
-      <color rgb="004472C4"/>
+      <color rgb="FF4472C4"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="游ゴシック"/>
+      <charset val="128"/>
+      <family val="3"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
@@ -51,23 +57,38 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-        <bgColor rgb="00FCE4D6"/>
+        <fgColor rgb="FFFCE4D6"/>
+        <bgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
-        <bgColor rgb="00D9E1F2"/>
+        <fgColor rgb="FFD9E1F2"/>
+        <bgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -82,7 +103,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -100,6 +121,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -509,8 +531,7 @@
     <col width="12" bestFit="1" customWidth="1" style="1" min="7" max="7"/>
     <col width="14" bestFit="1" customWidth="1" style="1" min="8" max="8"/>
     <col width="10" bestFit="1" customWidth="1" style="1" min="9" max="9"/>
-    <col width="12" bestFit="1" customWidth="1" style="1" min="10" max="10"/>
-    <col width="12" bestFit="1" customWidth="1" style="1" min="11" max="11"/>
+    <col width="12" bestFit="1" customWidth="1" style="1" min="10" max="11"/>
     <col width="15" bestFit="1" customWidth="1" style="1" min="12" max="12"/>
     <col width="20" bestFit="1" customWidth="1" style="1" min="13" max="13"/>
     <col width="22" bestFit="1" customWidth="1" style="1" min="14" max="14"/>
@@ -643,6 +664,36 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>refresh_document_list</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Refresh (導出値を更新)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>add_collection_sheet</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Add Collection Sheet</t>
+        </is>
+      </c>
+    </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>

</xml_diff>